<commit_message>
Adding Bind::type to C1, C2 and C3 to manage issues with string type.
</commit_message>
<xml_diff>
--- a/Demo/lf/demo_lf_tas_9999_2_part.xlsx
+++ b/Demo/lf/demo_lf_tas_9999_2_part.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\lf\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\07. Sightsavers\2025\Data related\DSA forms\Demo\lf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E41C1FB-C35C-4AB0-868D-22666FEB8C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43CACD52-816E-4026-81B7-7C6E47DBB7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="153">
   <si>
     <t>type</t>
   </si>
@@ -491,6 +491,9 @@
   </si>
   <si>
     <t>(Demo) 2. TAS1 LF Participant Form V2</t>
+  </si>
+  <si>
+    <t>bind::type</t>
   </si>
 </sst>
 </file>
@@ -1020,7 +1023,8 @@
     <col min="14" max="14" width="11" style="3"/>
     <col min="15" max="15" width="17.625" style="3" bestFit="1" customWidth="1"/>
     <col min="16" max="20" width="22.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="16384" width="11" style="3"/>
+    <col min="21" max="21" width="11.75" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="16384" width="11" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="4" customFormat="1" ht="37.5">
@@ -1086,6 +1090,9 @@
       </c>
       <c r="U1" s="1" t="s">
         <v>138</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:23" s="4" customFormat="1" ht="47.25">
@@ -1237,6 +1244,9 @@
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
+      <c r="V7" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="8" spans="1:23" s="4" customFormat="1">
       <c r="A8" s="15" t="s">
@@ -1280,6 +1290,9 @@
       <c r="K9" s="9"/>
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
+      <c r="V9" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="10" spans="1:23" s="4" customFormat="1">
       <c r="A10" s="9" t="s">
@@ -1301,6 +1314,9 @@
       <c r="K10" s="9"/>
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
+      <c r="V10" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="11" spans="1:23" s="4" customFormat="1">
       <c r="A11" s="4" t="s">

</xml_diff>

<commit_message>
added new demo forms
</commit_message>
<xml_diff>
--- a/Demo/lf/demo_lf_tas_9999_2_part.xlsx
+++ b/Demo/lf/demo_lf_tas_9999_2_part.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\lf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B1447BF-723C-49D6-8685-1C31038D2D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E6B8C0-1779-48AC-9C9B-B07465B13A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="206">
   <si>
     <t>type</t>
   </si>
@@ -637,6 +637,9 @@
   </si>
   <si>
     <t>${p_index_init} + indexed-repeat(${position}, ${p9999}, count(${p9999}))</t>
+  </si>
+  <si>
+    <t>Profession</t>
   </si>
 </sst>
 </file>
@@ -2237,7 +2240,7 @@
         <v>180</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
demo: updated the dashboard
</commit_message>
<xml_diff>
--- a/Demo/lf/demo_lf_tas_9999_2_part.xlsx
+++ b/Demo/lf/demo_lf_tas_9999_2_part.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\lf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E6B8C0-1779-48AC-9C9B-B07465B13A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E2E1098-C527-49BE-B519-5A0BC402F3E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -345,9 +345,6 @@
     <t>p_index_init</t>
   </si>
   <si>
-    <t>once(if(${last-saved#p_index_cur}!=null,${last-saved#p_index_cur, 0))</t>
-  </si>
-  <si>
     <t>Participant</t>
   </si>
   <si>
@@ -640,6 +637,9 @@
   </si>
   <si>
     <t>Profession</t>
+  </si>
+  <si>
+    <t>once(if(${last-saved#p_index_cur}!=null,${last-saved#p_index_cur}, 0))</t>
   </si>
 </sst>
 </file>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="2" spans="1:21" s="7" customFormat="1" ht="47.25">
       <c r="A2" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>78</v>
@@ -1340,10 +1340,10 @@
         <v>17</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D3" s="6"/>
       <c r="F3" s="27"/>
@@ -1367,10 +1367,10 @@
         <v>17</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D4" s="6"/>
       <c r="F4" s="27"/>
@@ -1384,7 +1384,7 @@
         <v>60</v>
       </c>
       <c r="Q4" s="28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
@@ -1396,10 +1396,10 @@
         <v>17</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D5" s="6"/>
       <c r="F5" s="27"/>
@@ -1413,7 +1413,7 @@
         <v>61</v>
       </c>
       <c r="R5" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S5" s="6"/>
       <c r="T5" s="6"/>
@@ -1424,10 +1424,10 @@
         <v>17</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D6" s="6"/>
       <c r="F6" s="27"/>
@@ -1443,7 +1443,7 @@
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
       <c r="S6" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="T6" s="6"/>
       <c r="U6" s="6"/>
@@ -1456,10 +1456,10 @@
         <v>94</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="E7" s="6"/>
       <c r="G7" s="6"/>
@@ -1475,13 +1475,13 @@
     </row>
     <row r="8" spans="1:21" s="7" customFormat="1" ht="94.5">
       <c r="A8" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>145</v>
-      </c>
       <c r="C8" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
@@ -1500,19 +1500,19 @@
     </row>
     <row r="9" spans="1:21" s="7" customFormat="1" ht="94.5">
       <c r="A9" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="6" t="s">
@@ -1550,7 +1550,7 @@
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
       <c r="I11" s="10" t="s">
-        <v>107</v>
+        <v>205</v>
       </c>
       <c r="J11" s="10"/>
       <c r="K11" s="10"/>
@@ -1602,10 +1602,10 @@
         <v>64</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D14" s="6"/>
       <c r="G14" s="6"/>
@@ -1725,7 +1725,7 @@
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
       <c r="H20" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I20" s="9" t="s">
         <v>105</v>
@@ -1754,10 +1754,10 @@
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
       <c r="H21" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="J21" s="9"/>
       <c r="K21" s="9"/>
@@ -1771,7 +1771,7 @@
         <v>50</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -1779,7 +1779,7 @@
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>67</v>
@@ -1809,17 +1809,17 @@
         <v>13</v>
       </c>
       <c r="B24" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C24" s="12" t="s">
         <v>113</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>114</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="12"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
       <c r="H24" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I24" s="12"/>
       <c r="J24" s="12" t="s">
@@ -1844,10 +1844,10 @@
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
       <c r="H25" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J25" s="12"/>
       <c r="K25" s="12"/>
@@ -1871,20 +1871,20 @@
     </row>
     <row r="27" spans="1:21" s="7" customFormat="1">
       <c r="A27" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>119</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>120</v>
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
       <c r="F27" s="14"/>
       <c r="G27" s="14"/>
       <c r="H27" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I27" s="14"/>
       <c r="J27" s="14" t="s">
@@ -1901,17 +1901,17 @@
         <v>87</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="14"/>
       <c r="G28" s="14"/>
       <c r="H28" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="14" t="s">
@@ -1928,17 +1928,17 @@
         <v>31</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
       <c r="F29" s="14"/>
       <c r="G29" s="14"/>
       <c r="H29" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I29" s="14"/>
       <c r="J29" s="14" t="s">
@@ -1955,21 +1955,21 @@
         <v>31</v>
       </c>
       <c r="B30" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" s="32" t="s">
         <v>126</v>
-      </c>
-      <c r="C30" s="32" t="s">
-        <v>127</v>
       </c>
       <c r="D30" s="32"/>
       <c r="E30" s="32"/>
       <c r="F30" s="32" t="s">
+        <v>129</v>
+      </c>
+      <c r="G30" s="32" t="s">
         <v>130</v>
       </c>
-      <c r="G30" s="32" t="s">
-        <v>131</v>
-      </c>
       <c r="H30" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I30" s="14"/>
       <c r="J30" s="32" t="s">
@@ -2002,7 +2002,7 @@
         <v>90</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="15"/>
@@ -2016,7 +2016,7 @@
         <v>95</v>
       </c>
       <c r="I32" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>16</v>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="O32" s="15"/>
       <c r="T32" s="28" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="U32" s="33" t="s">
         <v>63</v>
@@ -2071,10 +2071,10 @@
         <v>31</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -2096,10 +2096,10 @@
         <v>31</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -2121,10 +2121,10 @@
         <v>31</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
@@ -2134,7 +2134,7 @@
         <v>82</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J37" s="6" t="s">
         <v>16</v>
@@ -2159,7 +2159,7 @@
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
       <c r="F38" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>80</v>
@@ -2203,10 +2203,10 @@
         <v>18</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H40" s="7" t="s">
         <v>82</v>
@@ -2220,13 +2220,13 @@
         <v>31</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J41" s="8" t="s">
         <v>16</v>
@@ -2237,10 +2237,10 @@
         <v>31</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>82</v>
@@ -2251,13 +2251,13 @@
     </row>
     <row r="43" spans="1:14" ht="15.75" customHeight="1">
       <c r="A43" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H43" s="7"/>
     </row>
@@ -2289,7 +2289,7 @@
         <v>71</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J45" s="8" t="s">
         <v>16</v>
@@ -2300,13 +2300,13 @@
         <v>18</v>
       </c>
       <c r="B46" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="C46" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="C46" s="34" t="s">
-        <v>194</v>
-      </c>
       <c r="H46" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J46" s="8" t="s">
         <v>16</v>
@@ -2367,10 +2367,10 @@
         <v>18</v>
       </c>
       <c r="B49" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C49" s="6" t="s">
         <v>197</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>198</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
@@ -2392,10 +2392,10 @@
         <v>18</v>
       </c>
       <c r="B50" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C50" s="6" t="s">
         <v>199</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>200</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
@@ -2476,7 +2476,7 @@
         <v>50</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="9"/>
@@ -2487,7 +2487,7 @@
         <v>102</v>
       </c>
       <c r="I57" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J57" s="10"/>
       <c r="K57" s="10"/>
@@ -2624,7 +2624,7 @@
         <v>97</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2635,150 +2635,150 @@
         <v>101</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="C12" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="B17" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="B17" s="19" t="s">
-        <v>152</v>
-      </c>
       <c r="C17" s="20" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="21" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B21" s="19">
         <v>99</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>186</v>
-      </c>
       <c r="C23" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -2812,10 +2812,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C2" t="s">
         <v>48</v>

</xml_diff>